<commit_message>
validation: regenerate all outputs with real second-coder labels
generate_all_outputs.py now reads coder2_labels_full.csv when present
instead of running the seed=42 simulation, ensuring validation_results.xlsx,
kappa_agreement_detail.csv, and validation_report_data.json all reflect
the real independent kappa (0.568 three-label; 0.932 binary).

Also fix UnicodeEncodeError on Windows console (kappa symbol in print).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/validation/validation_results.xlsx
+++ b/validation/validation_results.xlsx
@@ -733,7 +733,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>82.4%</t>
+          <t>71.4%</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>0.7340</t>
+          <t>0.5684</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>[0.6183, 0.8457]</t>
+          <t>[0.4441, 0.6908]</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>82.4%</t>
+          <t>71.4%</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>0.7340</t>
+          <t>0.5684</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>[0.6183, 0.8457]</t>
+          <t>[0.4441, 0.6908]</t>
         </is>
       </c>
     </row>
@@ -1121,11 +1121,11 @@
         <v>20</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
     </row>
@@ -1157,11 +1157,11 @@
         <v>45</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>84.4%</t>
+          <t>86.7%</t>
         </is>
       </c>
     </row>
@@ -1219,13 +1219,13 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>33</v>
-      </c>
-      <c r="C20" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="11" t="n">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1234,11 +1234,11 @@
           <t>WATER</t>
         </is>
       </c>
-      <c r="B21" s="14" t="n">
-        <v>2</v>
+      <c r="B21" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D21" s="14" t="n">
         <v>3</v>
@@ -1251,13 +1251,13 @@
         </is>
       </c>
       <c r="B22" s="14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C22" s="14" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24">
@@ -1302,52 +1302,52 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>NOT_WATER</t>
+          <t>WATER</t>
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>0.846</t>
+          <t>0.562</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.900</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>WATER</t>
+          <t>NOT_WATER</t>
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C27" s="11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>0.781</t>
+          <t>0.968</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>0.833</t>
+          <t>0.909</t>
         </is>
       </c>
     </row>
@@ -1358,22 +1358,22 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>0.850</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>0.607</t>
+          <t>0.286</t>
         </is>
       </c>
     </row>
@@ -1495,18 +1495,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="b">
-        <v>1</v>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1759,18 +1759,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="b">
-        <v>1</v>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1825,18 +1825,18 @@
           <t>NL_plain</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>NOT_WATER</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="inlineStr">
-        <is>
-          <t>NOT_WATER</t>
-        </is>
-      </c>
-      <c r="G13" s="13" t="b">
-        <v>1</v>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>NOT_WATER</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2089,18 +2089,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>NOT_WATER</t>
-        </is>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
-        <is>
-          <t>NOT_WATER</t>
-        </is>
-      </c>
-      <c r="G21" s="13" t="b">
-        <v>1</v>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>NOT_WATER</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -2188,18 +2188,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="b">
-        <v>1</v>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -2386,18 +2386,18 @@
           <t>NL_broad_water</t>
         </is>
       </c>
-      <c r="E30" s="14" t="inlineStr">
-        <is>
-          <t>WATER</t>
-        </is>
-      </c>
-      <c r="F30" s="14" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G30" s="14" t="b">
-        <v>0</v>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>NOT_WATER</t>
+          <t>WATER</t>
         </is>
       </c>
       <c r="G34" s="14" t="b">
@@ -2551,18 +2551,18 @@
           <t>NL_broad_water</t>
         </is>
       </c>
-      <c r="E35" s="14" t="inlineStr">
-        <is>
-          <t>WATER</t>
-        </is>
-      </c>
-      <c r="F35" s="14" t="inlineStr">
-        <is>
-          <t>NOT_WATER</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="b">
-        <v>0</v>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -2716,18 +2716,18 @@
           <t>NL_plain</t>
         </is>
       </c>
-      <c r="E40" s="14" t="inlineStr">
+      <c r="E40" s="13" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F40" s="14" t="inlineStr">
-        <is>
-          <t>WATER</t>
-        </is>
-      </c>
-      <c r="G40" s="14" t="b">
-        <v>0</v>
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="F42" s="14" t="inlineStr">
         <is>
-          <t>NOT_WATER</t>
+          <t>WATER</t>
         </is>
       </c>
       <c r="G42" s="14" t="b">
@@ -2881,18 +2881,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr">
-        <is>
-          <t>NOT_WATER</t>
-        </is>
-      </c>
-      <c r="F45" s="13" t="inlineStr">
-        <is>
-          <t>NOT_WATER</t>
-        </is>
-      </c>
-      <c r="G45" s="13" t="b">
-        <v>1</v>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>NOT_WATER</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G45" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -2980,18 +2980,18 @@
           <t>NL_broad_water</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
-        <is>
-          <t>WATER</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="inlineStr">
-        <is>
-          <t>WATER</t>
-        </is>
-      </c>
-      <c r="G48" s="13" t="b">
-        <v>1</v>
+      <c r="E48" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="F48" s="14" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="G48" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -3442,18 +3442,18 @@
           <t>NL_broad_water</t>
         </is>
       </c>
-      <c r="E62" s="14" t="inlineStr">
-        <is>
-          <t>WATER</t>
-        </is>
-      </c>
-      <c r="F62" s="14" t="inlineStr">
-        <is>
-          <t>NOT_WATER</t>
-        </is>
-      </c>
-      <c r="G62" s="14" t="b">
-        <v>0</v>
+      <c r="E62" s="13" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G62" s="13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -3541,18 +3541,18 @@
           <t>NL_broad_water</t>
         </is>
       </c>
-      <c r="E65" s="13" t="inlineStr">
-        <is>
-          <t>WATER</t>
-        </is>
-      </c>
-      <c r="F65" s="13" t="inlineStr">
-        <is>
-          <t>WATER</t>
-        </is>
-      </c>
-      <c r="G65" s="13" t="b">
-        <v>1</v>
+      <c r="E65" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="F65" s="14" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="G65" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -3838,18 +3838,18 @@
           <t>NL_broad_water</t>
         </is>
       </c>
-      <c r="E74" s="14" t="inlineStr">
-        <is>
-          <t>WATER</t>
-        </is>
-      </c>
-      <c r="F74" s="14" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G74" s="14" t="b">
-        <v>0</v>
+      <c r="E74" s="13" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="F74" s="13" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G74" s="13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -3871,18 +3871,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E75" s="13" t="inlineStr">
+      <c r="E75" s="14" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F75" s="13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G75" s="13" t="b">
-        <v>1</v>
+      <c r="F75" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G75" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -3937,18 +3937,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E77" s="13" t="inlineStr">
+      <c r="E77" s="14" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F77" s="13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G77" s="13" t="b">
-        <v>1</v>
+      <c r="F77" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G77" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -4003,18 +4003,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E79" s="13" t="inlineStr">
+      <c r="E79" s="14" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F79" s="13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G79" s="13" t="b">
-        <v>1</v>
+      <c r="F79" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G79" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -4036,18 +4036,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E80" s="13" t="inlineStr">
+      <c r="E80" s="14" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F80" s="13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G80" s="13" t="b">
-        <v>1</v>
+      <c r="F80" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G80" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -4069,18 +4069,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E81" s="13" t="inlineStr">
+      <c r="E81" s="14" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F81" s="13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G81" s="13" t="b">
-        <v>1</v>
+      <c r="F81" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G81" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -4175,7 +4175,7 @@
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
-          <t>NOT_WATER</t>
+          <t>WATER</t>
         </is>
       </c>
       <c r="G84" s="14" t="b">
@@ -4234,18 +4234,18 @@
           <t>NL_broad_water</t>
         </is>
       </c>
-      <c r="E86" s="13" t="inlineStr">
+      <c r="E86" s="14" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F86" s="13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G86" s="13" t="b">
-        <v>1</v>
+      <c r="F86" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G86" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -4366,18 +4366,18 @@
           <t>BR_all</t>
         </is>
       </c>
-      <c r="E90" s="13" t="inlineStr">
+      <c r="E90" s="14" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
       </c>
-      <c r="F90" s="13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="G90" s="13" t="b">
-        <v>1</v>
+      <c r="F90" s="14" t="inlineStr">
+        <is>
+          <t>WATER</t>
+        </is>
+      </c>
+      <c r="G90" s="14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="91">

</xml_diff>